<commit_message>
chore: update FX rates (2026-06-06 23:19 UTC)
</commit_message>
<xml_diff>
--- a/data/sample_input.xlsx
+++ b/data/sample_input.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -444,6 +444,21 @@
           <t>description</t>
         </is>
       </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>live_rate</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>converted_try</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>last_updated</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -459,6 +474,17 @@
           <t>Laptop</t>
         </is>
       </c>
+      <c r="D2" t="n">
+        <v>46.084</v>
+      </c>
+      <c r="E2" t="n">
+        <v>460.84</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>2026-06-06 23:19 UTC</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -474,6 +500,17 @@
           <t>Travel</t>
         </is>
       </c>
+      <c r="D3" t="n">
+        <v>53.64155928810047</v>
+      </c>
+      <c r="E3" t="n">
+        <v>268.2077964405024</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2026-06-06 23:19 UTC</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -487,6 +524,17 @@
       <c r="C4" t="inlineStr">
         <is>
           <t>Coffee</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" t="n">
+        <v>100</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2026-06-06 23:19 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>